<commit_message>
admin workload overview and overload warning
</commit_message>
<xml_diff>
--- a/docs/ProductBacklog_group51.xlsx
+++ b/docs/ProductBacklog_group51.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\庄天婧\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Recruitment-System-for-TA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D5BDC4-68A6-48BB-8672-A5BA3E89E0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6F69B1-95C4-4AED-9756-F24708A41AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -579,68 +579,73 @@
 3. Warning displayed if workload exceeds limit</t>
   </si>
   <si>
+    <t>Balance TA workload</t>
+  </si>
+  <si>
+    <t>Manage users</t>
+  </si>
+  <si>
+    <t>As an administrator
+I want to manage user accounts
+So that I can maintain system security and integrity.</t>
+  </si>
+  <si>
+    <t>1. Admin can view list of users
+2. Admin can deactivate or delete user accounts
+3. Admin can view user roles</t>
+  </si>
+  <si>
+    <t>Manage job postings</t>
+  </si>
+  <si>
+    <t>As an administrator
+I want to manage job postings
+So that inappropriate or outdated jobs can be removed.</t>
+  </si>
+  <si>
+    <t>1. Admin can view all job postings
+2. Admin can edit job information
+3. Admin can delete job postings</t>
+  </si>
+  <si>
+    <t>US-32</t>
+  </si>
+  <si>
+    <t>Export recruitment data</t>
+  </si>
+  <si>
+    <t>As an administrator
+I want to export recruitment data
+So that I can analyze recruitment results externally.</t>
+  </si>
+  <si>
+    <t>1. Admin can export applicant data
+2. Admin can export job application records
+3. Data can be exported as CSV or Excel file</t>
+  </si>
+  <si>
     <t>US-29</t>
-  </si>
-  <si>
-    <t>Balance TA workload</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>US-30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>US-31</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. System calculates workload of each TA
+2. TAs with lower workload are highlighted
+3. Recommendations appear when MO assigning jobs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>As an administrator
 I want the system to recommend TAs with lower workload
 So that tasks can be distributed more fairly.</t>
-  </si>
-  <si>
-    <t>1. System calculates workload of each TA
-2. TAs with lower workload are highlighted
-3. Recommendations appear when assigning jobs</t>
-  </si>
-  <si>
-    <t>US-30</t>
-  </si>
-  <si>
-    <t>Manage users</t>
-  </si>
-  <si>
-    <t>As an administrator
-I want to manage user accounts
-So that I can maintain system security and integrity.</t>
-  </si>
-  <si>
-    <t>1. Admin can view list of users
-2. Admin can deactivate or delete user accounts
-3. Admin can view user roles</t>
-  </si>
-  <si>
-    <t>US-31</t>
-  </si>
-  <si>
-    <t>Manage job postings</t>
-  </si>
-  <si>
-    <t>As an administrator
-I want to manage job postings
-So that inappropriate or outdated jobs can be removed.</t>
-  </si>
-  <si>
-    <t>1. Admin can view all job postings
-2. Admin can edit job information
-3. Admin can delete job postings</t>
-  </si>
-  <si>
-    <t>US-32</t>
-  </si>
-  <si>
-    <t>Export recruitment data</t>
-  </si>
-  <si>
-    <t>As an administrator
-I want to export recruitment data
-So that I can analyze recruitment results externally.</t>
-  </si>
-  <si>
-    <t>1. Admin can export applicant data
-2. Admin can export job application records
-3. Data can be exported as CSV or Excel file</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -650,7 +655,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -668,6 +673,14 @@
     <font>
       <sz val="9"/>
       <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -718,7 +731,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -738,6 +751,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1229,7 +1251,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr defaultColWidth="9.81640625" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.81640625" style="4"/>
@@ -2118,9 +2140,9 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="84" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>136</v>
+    <row r="30" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>147</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>137</v>
@@ -2129,7 +2151,7 @@
         <v>138</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="E30" s="4">
         <v>2</v>
@@ -2138,7 +2160,7 @@
         <v>139</v>
       </c>
       <c r="G30" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I30" s="6">
         <v>46117</v>
@@ -2147,24 +2169,24 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:10" ht="64" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="C31" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E31" s="4">
+        <v>2</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>142</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" s="4">
-        <v>2</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="G31" s="4">
         <v>3</v>
@@ -2176,24 +2198,24 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="64" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="70" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E32" s="4">
+        <v>3</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E32" s="4">
-        <v>2</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>147</v>
       </c>
       <c r="G32" s="4">
         <v>3</v>
@@ -2205,47 +2227,46 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="70" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>148</v>
+    <row r="33" spans="1:10" ht="84" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>149</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C33" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E33" s="4">
+        <v>2</v>
+      </c>
+      <c r="F33" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E33" s="4">
-        <v>3</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>151</v>
-      </c>
       <c r="G33" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I33" s="6">
         <v>46125</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="9">
         <v>46138</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="112" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:10" ht="104" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:10" ht="103" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:10" ht="86" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:10" ht="79" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:10" ht="73" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:10" ht="92" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C47" s="5"/>
-      <c r="F47" s="5"/>
+    <row r="34" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="1:10" ht="104" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:10" ht="103" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:10" ht="86" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:10" ht="79" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:10" ht="73" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:10" ht="92" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C46" s="5"/>
+      <c r="F46" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
force the status to change
</commit_message>
<xml_diff>
--- a/docs/ProductBacklog_group51.xlsx
+++ b/docs/ProductBacklog_group51.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Github\Recruitment-System-for-TA\docs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD28E738-D420-458F-882B-5585B1A54C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="24750" windowHeight="10480"/>
   </bookViews>
   <sheets>
     <sheet name="ProductBacklog_group51" sheetId="1" r:id="rId1"/>
@@ -24,6 +18,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -31,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="164">
   <si>
     <t>Story ID</t>
   </si>
@@ -394,6 +390,39 @@
     <t>US-19</t>
   </si>
   <si>
+    <t>Save favorite jobs</t>
+  </si>
+  <si>
+    <t>As a TA applicant
+I want to save jobs as favorites
+So that I can review them later easily.</t>
+  </si>
+  <si>
+    <t>1. User can click "Save" on a job
+2. Saved jobs are stored (JSON is OK)
+3. User can view a list of saved jobs
+4. User can remove a saved job</t>
+  </si>
+  <si>
+    <t>US-20</t>
+  </si>
+  <si>
+    <t>View recently viewed jobs</t>
+  </si>
+  <si>
+    <t>As a TA applicant
+I want to see recently viewed jobs
+So that I can easily revisit them.</t>
+  </si>
+  <si>
+    <t>1. System stores recently viewed jobs
+2. User can view list of recent jobs
+3. List is limited (e.g., last 5 jobs)</t>
+  </si>
+  <si>
+    <t>US-21</t>
+  </si>
+  <si>
     <t>Apply for job</t>
   </si>
   <si>
@@ -407,7 +436,7 @@
 3. Confirmation message is displayed</t>
   </si>
   <si>
-    <t>US-20</t>
+    <t>US-22</t>
   </si>
   <si>
     <t>Check application status</t>
@@ -423,7 +452,10 @@
 3. Status updates when MO makes decision</t>
   </si>
   <si>
-    <t>US-21</t>
+    <t>US-23</t>
+  </si>
+  <si>
+    <t>Applications Manage</t>
   </si>
   <si>
     <t>As a TA applicant
@@ -436,7 +468,10 @@
 3. Reorder: User can change the preference order of applications</t>
   </si>
   <si>
-    <t>US-22</t>
+    <t>Essential for the algorithm to resolve multiple offers</t>
+  </si>
+  <si>
+    <t>US-24</t>
   </si>
   <si>
     <t>Identify missing skills</t>
@@ -452,7 +487,7 @@
 3. Suggestions are displayed</t>
   </si>
   <si>
-    <t>US-23</t>
+    <t>US-25</t>
   </si>
   <si>
     <t>AI Job Recommendation</t>
@@ -471,7 +506,7 @@
     <t>AI recommendation feature</t>
   </si>
   <si>
-    <t>US-24</t>
+    <t>US-26</t>
   </si>
   <si>
     <t>Post job</t>
@@ -492,7 +527,7 @@
 8. MO can click Publish to make the vacancy visible to students.</t>
   </si>
   <si>
-    <t>US-25</t>
+    <t>US-27</t>
   </si>
   <si>
     <t>Select applicants</t>
@@ -516,7 +551,7 @@
 11. MO can notify the selected applicant via email or in the system (if email integration is available).</t>
   </si>
   <si>
-    <t>US-26</t>
+    <t>US-28</t>
   </si>
   <si>
     <t>View Applicant List</t>
@@ -538,7 +573,7 @@
 9. MO can click on an applicant's name to view the full profile.</t>
   </si>
   <si>
-    <t>US-27</t>
+    <t>US-29</t>
   </si>
   <si>
     <t>Skill matching</t>
@@ -555,7 +590,7 @@
 4. MO can click on the matching result to view more detailed reasoning behind the match.</t>
   </si>
   <si>
-    <t>US-28</t>
+    <t>US-30</t>
   </si>
   <si>
     <t>View TA workload</t>
@@ -571,7 +606,7 @@
 3. Warning displayed if workload exceeds limit</t>
   </si>
   <si>
-    <t>US-29</t>
+    <t>US-31</t>
   </si>
   <si>
     <t>Balance TA workload</t>
@@ -582,7 +617,12 @@
 So that tasks can be distributed more fairly.</t>
   </si>
   <si>
-    <t>US-30</t>
+    <t>1. System calculates workload of each TA
+2. TAs with lower workload are highlighted
+3. Recommendations appear when MO assigns jobs</t>
+  </si>
+  <si>
+    <t>US-32</t>
   </si>
   <si>
     <t>Manage users</t>
@@ -598,7 +638,7 @@
 3. Admin can view user roles</t>
   </si>
   <si>
-    <t>US-31</t>
+    <t>US-33</t>
   </si>
   <si>
     <t>Manage job postings</t>
@@ -614,7 +654,10 @@
 3. Admin can delete job postings</t>
   </si>
   <si>
-    <t>US-32</t>
+    <t>US-34</t>
+  </si>
+  <si>
+    <t>Export recruitment data</t>
   </si>
   <si>
     <t>As an administrator
@@ -627,71 +670,36 @@
 3. Data can be exported as CSV or Excel file</t>
   </si>
   <si>
-    <t>Applications Manage</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Essential for the algorithm to resolve multiple offers</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Export recruitment data</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. System calculates workload of each TA
-2. TAs with lower workload are highlighted
-3. Recommendations appear when MO assigns jobs</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>US-33</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Save favorite jobs</t>
-  </si>
-  <si>
-    <t>As a TA applicant
-I want to save jobs as favorites
-So that I can review them later easily.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. User can click "Save" on a job
-2. Saved jobs are stored (JSON is OK)
-3. User can view a list of saved jobs
-4. User can remove a saved job</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>View recently viewed jobs</t>
-  </si>
-  <si>
-    <t>As a TA applicant
-I want to see recently viewed jobs
-So that I can easily revisit them.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Should</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. System stores recently viewed jobs
-2. User can view list of recent jobs
-3. List is limited (e.g., last 5 jobs)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <t>US-35</t>
+  </si>
+  <si>
+    <t>Override application status</t>
+  </si>
+  <si>
+    <t>As an administrator
+I want to force-change TA application status from the status-filtered lists
+So that I can correct or override MO decisions when needed.</t>
+  </si>
+  <si>
+    <t>1. On the Pending list, admin can Force accept or Force reject each application.
+2. On the Accepted list, admin can Force reject or Force pend.
+3. On the Rejected list, admin can Force accept or Force pend.
+4. Status updates are persisted the same way as normal workflow.
+5. After an action, admin sees feedback on the list page.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -703,25 +711,155 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
-      <family val="3"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -730,12 +868,192 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -758,12 +1076,251 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -777,181 +1334,111 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="27" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="2" borderId="1" xfId="27" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="40% - 着色 1" xfId="1" builtinId="31"/>
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
       <border>
@@ -962,7 +1449,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -990,40 +1477,154 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
+          <color theme="4" tint="0.399975585192419"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="16"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="totalRow" dxfId="14"/>
-      <tableStyleElement type="firstColumn" dxfId="13"/>
-      <tableStyleElement type="lastColumn" dxfId="12"/>
-      <tableStyleElement type="firstRowStripe" dxfId="11"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
-      <tableStyleElement type="pageFieldValues" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1281,25 +1882,25 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:J47"/>
-  <sheetFormatPr defaultColWidth="9.796875" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.8" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="9.796875" style="1"/>
-    <col min="2" max="2" width="13.59765625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="33.59765625" style="1" customWidth="1"/>
-    <col min="4" max="5" width="9.796875" style="1"/>
-    <col min="6" max="6" width="39.33203125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="9.796875" style="1"/>
-    <col min="9" max="10" width="12.19921875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.8" style="1"/>
+    <col min="2" max="2" width="13.6" style="1" customWidth="1"/>
+    <col min="3" max="3" width="33.6" style="1" customWidth="1"/>
+    <col min="4" max="5" width="9.8" style="1"/>
+    <col min="6" max="6" width="39.3363636363636" style="1" customWidth="1"/>
+    <col min="7" max="8" width="9.8" style="1"/>
+    <col min="9" max="10" width="12.2" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+    <row r="1" ht="56" spans="1:10">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1331,7 +1932,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+    <row r="2" ht="84" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1363,7 +1964,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+    <row r="3" ht="84" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -1395,7 +1996,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+    <row r="4" ht="56" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1427,7 +2028,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+    <row r="5" ht="84" spans="1:10">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -1459,7 +2060,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="6" ht="70" spans="1:10">
       <c r="A6" s="1" t="s">
         <v>31</v>
       </c>
@@ -1491,7 +2092,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="7" ht="70" spans="1:10">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -1523,7 +2124,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+    <row r="8" ht="84" spans="1:10">
       <c r="A8" s="1" t="s">
         <v>42</v>
       </c>
@@ -1552,7 +2153,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" ht="87" customHeight="1" spans="1:10">
       <c r="A9" s="1" t="s">
         <v>46</v>
       </c>
@@ -1581,7 +2182,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" ht="70.05" customHeight="1" spans="1:10">
       <c r="A10" s="1" t="s">
         <v>50</v>
       </c>
@@ -1610,7 +2211,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+    <row r="11" ht="56" spans="1:10">
       <c r="A11" s="1" t="s">
         <v>54</v>
       </c>
@@ -1639,7 +2240,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="110" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" ht="110" customHeight="1" spans="1:10">
       <c r="A12" s="1" t="s">
         <v>59</v>
       </c>
@@ -1668,7 +2269,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="13" ht="98" spans="1:10">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1697,7 +2298,7 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="92" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" ht="92" customHeight="1" spans="1:10">
       <c r="A14" s="1" t="s">
         <v>67</v>
       </c>
@@ -1726,7 +2327,7 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+    <row r="15" ht="56" spans="1:10">
       <c r="A15" s="1" t="s">
         <v>71</v>
       </c>
@@ -1755,7 +2356,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="138" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" ht="138" customHeight="1" spans="1:10">
       <c r="A16" s="1" t="s">
         <v>75</v>
       </c>
@@ -1784,7 +2385,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="118.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" ht="118.05" customHeight="1" spans="1:10">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1816,7 +2417,7 @@
         <v>46130</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="18" ht="98" spans="1:10">
       <c r="A18" s="1" t="s">
         <v>84</v>
       </c>
@@ -1848,7 +2449,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" ht="81" customHeight="1" spans="1:10">
       <c r="A19" s="1" t="s">
         <v>89</v>
       </c>
@@ -1880,24 +2481,24 @@
         <v>46130</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" ht="63" customHeight="1" spans="1:10">
       <c r="A20" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>153</v>
+      <c r="B20" s="6" t="s">
+        <v>95</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="D20" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="1">
         <v>3</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>155</v>
+        <v>97</v>
       </c>
       <c r="G20" s="1">
         <v>3</v>
@@ -1909,24 +2510,24 @@
         <v>46144</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="21" ht="70" spans="1:10">
       <c r="A21" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>156</v>
+      <c r="B21" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>158</v>
+        <v>100</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>34</v>
       </c>
       <c r="E21" s="1">
         <v>4</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>159</v>
+        <v>101</v>
       </c>
       <c r="G21" s="1">
         <v>2</v>
@@ -1938,15 +2539,15 @@
         <v>46158</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+    <row r="22" ht="56" spans="1:10">
       <c r="A22" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>13</v>
@@ -1955,7 +2556,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="G22" s="1">
         <v>5</v>
@@ -1967,15 +2568,15 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+    <row r="23" ht="84" spans="1:10">
       <c r="A23" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>34</v>
@@ -1984,7 +2585,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="G23" s="1">
         <v>3</v>
@@ -1996,15 +2597,15 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="24" ht="98" spans="1:10">
       <c r="A24" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>148</v>
+        <v>110</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>111</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>34</v>
@@ -2013,13 +2614,13 @@
         <v>2</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="G24" s="1">
         <v>3</v>
       </c>
-      <c r="H24" s="6" t="s">
-        <v>149</v>
+      <c r="H24" s="9" t="s">
+        <v>114</v>
       </c>
       <c r="I24" s="2">
         <v>46118</v>
@@ -2028,15 +2629,15 @@
         <v>46127</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="25" ht="70" spans="1:10">
       <c r="A25" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>57</v>
@@ -2045,7 +2646,7 @@
         <v>3</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="G25" s="1">
         <v>8</v>
@@ -2057,15 +2658,15 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="26" ht="70" spans="1:10">
       <c r="A26" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>57</v>
@@ -2074,13 +2675,13 @@
         <v>3</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="G26" s="1">
         <v>5</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="I26" s="2">
         <v>46117</v>
@@ -2089,15 +2690,15 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="216" x14ac:dyDescent="0.3">
+    <row r="27" ht="224" spans="1:10">
       <c r="A27" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>13</v>
@@ -2106,7 +2707,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G27" s="1">
         <v>5</v>
@@ -2118,15 +2719,15 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="351" x14ac:dyDescent="0.3">
+    <row r="28" ht="364" spans="1:10">
       <c r="A28" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>13</v>
@@ -2135,7 +2736,7 @@
         <v>2</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="G28" s="1">
         <v>5</v>
@@ -2147,15 +2748,15 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" ht="75" customHeight="1" spans="1:10">
       <c r="A29" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>13</v>
@@ -2164,7 +2765,7 @@
         <v>2</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="G29" s="1">
         <v>5</v>
@@ -2176,24 +2777,24 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="162" x14ac:dyDescent="0.3">
+    <row r="30" ht="168" spans="1:10">
       <c r="A30" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E30" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G30" s="1">
         <v>5</v>
@@ -2205,15 +2806,15 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" ht="105" customHeight="1" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>34</v>
@@ -2222,7 +2823,7 @@
         <v>2</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="G31" s="1">
         <v>3</v>
@@ -2234,24 +2835,24 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="64.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" ht="64.05" customHeight="1" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>34</v>
       </c>
       <c r="E32" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="G32" s="1">
         <v>5</v>
@@ -2263,24 +2864,24 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+    <row r="33" ht="56" spans="1:10">
       <c r="A33" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E33" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="G33" s="1">
         <v>3</v>
@@ -2292,24 +2893,24 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="112.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
+    <row r="34" ht="112.05" customHeight="1" spans="1:10">
+      <c r="A34" s="9" t="s">
         <v>152</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="G34" s="1">
         <v>3</v>
@@ -2321,21 +2922,24 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="6" t="s">
-        <v>150</v>
+    <row r="35" ht="87" customHeight="1" spans="1:10">
+      <c r="A35" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>157</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E35" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="G35" s="1">
         <v>3</v>
@@ -2347,19 +2951,50 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="104" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:10" ht="103.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" spans="1:10" ht="86" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="1:10" ht="79.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="1:10" ht="73.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="1:10" ht="92" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" ht="104" customHeight="1" spans="1:10">
+      <c r="A36" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="1">
+        <v>4</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="G36" s="5">
+        <v>3</v>
+      </c>
+      <c r="I36" s="2">
+        <v>46139</v>
+      </c>
+      <c r="J36" s="2">
+        <v>46158</v>
+      </c>
+    </row>
+    <row r="37" ht="103.05" customHeight="1" spans="1:10">
+      <c r="G37" s="5"/>
+      <c r="I37" s="5"/>
+    </row>
+    <row r="38" ht="86" customHeight="1"/>
+    <row r="39" ht="79.05" customHeight="1"/>
+    <row r="40" ht="87" customHeight="1"/>
+    <row r="41" ht="73.05" customHeight="1"/>
+    <row r="42" ht="92" customHeight="1"/>
+    <row r="47" spans="1:10">
       <c r="C47" s="5"/>
       <c r="F47" s="5"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>